<commit_message>
Add Demand Planner roles sheet to job_listings_v2.xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job_listings_v2.xlsx
+++ b/job_listings_v2.xlsx
@@ -10,6 +10,7 @@
     <sheet name="o9 OMP Roles" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Supply Chain Architect Roles" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="🔥 Last 24 Hours" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Demand Planner Roles" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +56,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +95,11 @@
         <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -115,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -143,6 +155,24 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1363,4 +1393,453 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Demand Planner / Senior Demand Planner Roles — US Job Listings</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="8" customHeight="1"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Job Title</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Recruiter / HM</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Sr. Supply Demand Planner ⭐</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Intuitive</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Sunnyvale, CA</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>On-site · Full-time</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>$118.7K–$170.7K</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>2 o9 alumni work here · Responses managed off LinkedIn</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Sr. Supply &amp; Demand Planner ⭐</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Kohler Co.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Kohler, WI</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>On-site · Full-time</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Taylor Magri, CRD
+Recruiter @ Kohler</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>o9 alumni in network · Message recruiter directly!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Senior Supply Chain Planner ⭐</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Micron Technology</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Boise, ID</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>On-site · Full-time</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>50 school alumni work here</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Senior Analyst, Supply Chain Planning ⭐</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Analog Devices</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Wilmington, MA</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>140 school alumni work here</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Supply Chain Analysts – Sr #GA001 ⭐</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Cummins Inc.</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>On-site · Full-time</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>73 school alumni work here</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Sr Demand Planner (Ecomm &amp; Wholesale) 🟢</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Velvet Caviar</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>New York, US</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>$90K–$120K</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Easy Apply · Actively reviewing applicants</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Senior S&amp;OP Planner</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>On-site · Full-time</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>11 o9 alumni work here</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId7"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intel Senior Demand Planner roles (Santa Clara + Folsom) to Demand Planner sheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job_listings_v2.xlsx
+++ b/job_listings_v2.xlsx
@@ -1401,7 +1401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1827,6 +1827,106 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Senior Demand Planner ⭐</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Santa Clara, CA</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Rutvi (in network)</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>381 school alumni · Mentions Blue Yonder! · Responses managed off LinkedIn · 4 days ago</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Senior Demand Planner ⭐</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Folsom, CA</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Rutvi (in network)</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>381 school alumni · Mentions Blue Yonder! · Responses managed off LinkedIn · 4 days ago</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -1839,6 +1939,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Deloitte supply chain & planning roles sheet (Sheet 5)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job_listings_v2.xlsx
+++ b/job_listings_v2.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Supply Chain Architect Roles" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="🔥 Last 24 Hours" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Demand Planner Roles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="🏢 Deloitte Roles" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +63,26 @@
       <color rgb="00375623"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00004B23"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +119,21 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0086BC25"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00004B23"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF5E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -172,6 +206,36 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1944,4 +2008,506 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>🏢 Deloitte — Supply Chain &amp; Planning Roles — US Job Listings</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="8" customHeight="1"/>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Job Title</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="H3" s="17" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>Apply Deadline</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>Supply Chain Planning Manager ⭐⭐
+(o9, OMP, or Blue Yonder/JDA)</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Charlotte, NC + Multiple</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>PERFECT</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>8+ yrs SC · o9/OMP/BY in title! · S&amp;OP/IBP · 50% travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Supply Chain Planning Senior Consultant ⭐⭐
+(o9, OMP, or Blue Yonder/JDA)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Huntsville, AL (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>$95K–$135K est.</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>PERFECT</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>5+ yrs SC · o9/OMP/BY in title! · Demand/Supply/Inventory Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Supply Chain Planning Consultant ⭐
+(o9, OMP, or Blue Yonder/JDA)</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Huntsville, AL (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>$67K–$111K est.</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Open · 1 wk ago</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>3+ yrs SC · o9/OMP/BY in title! · Entry to Senior Consultant level</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>SCNO Strategic Sourcing &amp; Procurement Senior Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Charlotte, NC (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>$159K–$293K 💰</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>5/30/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>28 o9 alumni · 2 days ago · Coupa/Ariba/iValua · SC transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>SCNO Strategic Sourcing &amp; Procurement Senior Manager ⭐</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Atlanta, GA (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>$159K–$293K 💰</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>STRONG</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>5/30/2026</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>28 o9 alumni · 2 days ago · Same role different location</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Supply Chain Sourcing &amp; Procurement Consulting Manager</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>New York, NY (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>$130.8K–$241K 💰</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Open · 4 days ago</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>28 o9 alumni · Coupa/Ariba/iValua · Category Mgmt · 50% travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Supply Chain Sourcing &amp; Procurement Consulting Manager</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>$130.8K–$241K 💰</t>
+        </is>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>Open · 4 days ago</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>28 o9 alumni · Same role, Philly location</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Supply Chain Manager</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Jersey City, NJ (Hybrid)</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Hybrid · Full-time</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>View Job →</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Open · 1 wk ago</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>28 o9 alumni · Oracle SC Cloud · Be an early applicant</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId8"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>